<commit_message>
Switch radio baseline to 2.4 GHz (all teams): E01-ML01DP5, 250 kbps, two FR4 patches
- linkbudget.py: E01-ML01DP5 profile (+7 dBm est., pad to 10 dBm e.i.r.p., 4.5 dBi patch),
  scenarios S16-S20 (SRI/MRM/NM baseline, 1 Mbps SRI, 100 mW FHSS what-if), MRM near-far
  and channel-plan printout (nRF24 C/I at 250 kbps, RF_CH 24/49/74/82)
- build_workbook.py + xlsx: per-scenario BW/NF, UN-85 a) FHSS limit, E01 candidates rows;
  formulas recalculated, 0 difference vs Python
- DECISIONS.md: D-R1b band, D-R2b module, D-R4 draft channel plan, D-R5b patches;
  868 MHz records marked superseded
- ATENEA_QUESTIONS.md: Q2 obsolete, Q3 (FHSS 100 mW) and Q4 rewritten, Q10 two antennas
- CLAUDE.md: status + session log for the band switch

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U9KKjceZdEFpkWHQjWd6RY
</commit_message>
<xml_diff>
--- a/radio/MTP-F26_TeamC_Radio_LinkBudget.xlsx
+++ b/radio/MTP-F26_TeamC_Radio_LinkBudget.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Link Budget" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Height Sweep" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Throughput" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidates" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regulatory" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Link Budget" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Height Sweep" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Throughput" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Candidates" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Regulatory" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -721,7 +721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S76"/>
+  <dimension ref="A1:X81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -743,6 +743,11 @@
     <col width="17" customWidth="1" min="17" max="17"/>
     <col width="17" customWidth="1" min="18" max="18"/>
     <col width="17" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="17" customWidth="1" min="21" max="21"/>
+    <col width="17" customWidth="1" min="22" max="22"/>
+    <col width="17" customWidth="1" min="23" max="23"/>
+    <col width="17" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -853,6 +858,31 @@
       <c r="S3" s="5" t="inlineStr">
         <is>
           <t>S15</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>S17</t>
+        </is>
+      </c>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
+          <t>S18</t>
+        </is>
+      </c>
+      <c r="W3" s="5" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="X3" s="5" t="inlineStr">
+        <is>
+          <t>S20</t>
         </is>
       </c>
     </row>
@@ -880,6 +910,11 @@
       <c r="Q4" s="7" t="n"/>
       <c r="R4" s="7" t="n"/>
       <c r="S4" s="7" t="n"/>
+      <c r="T4" s="7" t="n"/>
+      <c r="U4" s="7" t="n"/>
+      <c r="V4" s="7" t="n"/>
+      <c r="W4" s="7" t="n"/>
+      <c r="X4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -967,6 +1002,31 @@
       <c r="S5" s="8" t="inlineStr">
         <is>
           <t>Bench 70 m</t>
+        </is>
+      </c>
+      <c r="T5" s="8" t="inlineStr">
+        <is>
+          <t>SRI 70 m</t>
+        </is>
+      </c>
+      <c r="U5" s="8" t="inlineStr">
+        <is>
+          <t>SRI 70 m</t>
+        </is>
+      </c>
+      <c r="V5" s="8" t="inlineStr">
+        <is>
+          <t>MRM 260 m</t>
+        </is>
+      </c>
+      <c r="W5" s="8" t="inlineStr">
+        <is>
+          <t>NM hop 100 m</t>
+        </is>
+      </c>
+      <c r="X5" s="8" t="inlineStr">
+        <is>
+          <t>MRM 260 m</t>
         </is>
       </c>
     </row>
@@ -1054,6 +1114,31 @@
           <t>RFM69HCW 869.85 | 100 kbps, +9 dBm (BENCH_5MW)</t>
         </is>
       </c>
+      <c r="T6" s="8" t="inlineStr">
+        <is>
+          <t>E01-ML01DP5 2.4G | 250 kbps, patches (2.4 baseline)</t>
+        </is>
+      </c>
+      <c r="U6" s="8" t="inlineStr">
+        <is>
+          <t>E01-ML01DP5 2.4G | 1 Mbps, patches</t>
+        </is>
+      </c>
+      <c r="V6" s="8" t="inlineStr">
+        <is>
+          <t>E01-ML01DP5 2.4G | 250 kbps, patches (2.4 baseline)</t>
+        </is>
+      </c>
+      <c r="W6" s="8" t="inlineStr">
+        <is>
+          <t>E01-ML01DP5 2.4G | 250 kbps, -10 dB obstr. (2.4 baseline)</t>
+        </is>
+      </c>
+      <c r="X6" s="8" t="inlineStr">
+        <is>
+          <t>E01-ML01DP5 2.4G | 250 kbps, 100 mW FHSS (if Atenea Q3 = yes)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1120,6 +1205,21 @@
       </c>
       <c r="S7" s="9" t="n">
         <v>100</v>
+      </c>
+      <c r="T7" s="9" t="n">
+        <v>250</v>
+      </c>
+      <c r="U7" s="9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="V7" s="9" t="n">
+        <v>250</v>
+      </c>
+      <c r="W7" s="9" t="n">
+        <v>250</v>
+      </c>
+      <c r="X7" s="9" t="n">
+        <v>250</v>
       </c>
     </row>
     <row r="8">
@@ -1210,6 +1310,31 @@
           <t>ERP</t>
         </is>
       </c>
+      <c r="T8" s="10" t="inlineStr">
+        <is>
+          <t>EIRP</t>
+        </is>
+      </c>
+      <c r="U8" s="10" t="inlineStr">
+        <is>
+          <t>EIRP</t>
+        </is>
+      </c>
+      <c r="V8" s="10" t="inlineStr">
+        <is>
+          <t>EIRP</t>
+        </is>
+      </c>
+      <c r="W8" s="10" t="inlineStr">
+        <is>
+          <t>EIRP</t>
+        </is>
+      </c>
+      <c r="X8" s="10" t="inlineStr">
+        <is>
+          <t>EIRP</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1276,6 +1401,21 @@
       </c>
       <c r="S9" s="11" t="n">
         <v>7</v>
+      </c>
+      <c r="T9" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="U9" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="V9" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="W9" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="X9" s="11" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -1302,6 +1442,11 @@
       <c r="Q10" s="7" t="n"/>
       <c r="R10" s="7" t="n"/>
       <c r="S10" s="7" t="n"/>
+      <c r="T10" s="7" t="n"/>
+      <c r="U10" s="7" t="n"/>
+      <c r="V10" s="7" t="n"/>
+      <c r="W10" s="7" t="n"/>
+      <c r="X10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1369,6 +1514,21 @@
       <c r="S11" s="12" t="n">
         <v>869.85</v>
       </c>
+      <c r="T11" s="12" t="n">
+        <v>2440</v>
+      </c>
+      <c r="U11" s="12" t="n">
+        <v>2440</v>
+      </c>
+      <c r="V11" s="12" t="n">
+        <v>2440</v>
+      </c>
+      <c r="W11" s="12" t="n">
+        <v>2440</v>
+      </c>
+      <c r="X11" s="12" t="n">
+        <v>2441</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1436,6 +1596,21 @@
       <c r="S12" s="13" t="n">
         <v>299792458</v>
       </c>
+      <c r="T12" s="13" t="n">
+        <v>299792458</v>
+      </c>
+      <c r="U12" s="13" t="n">
+        <v>299792458</v>
+      </c>
+      <c r="V12" s="13" t="n">
+        <v>299792458</v>
+      </c>
+      <c r="W12" s="13" t="n">
+        <v>299792458</v>
+      </c>
+      <c r="X12" s="13" t="n">
+        <v>299792458</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1516,6 +1691,26 @@
       </c>
       <c r="S13" s="14">
         <f>S12/(S11*1000000)</f>
+        <v/>
+      </c>
+      <c r="T13" s="14">
+        <f>T12/(T11*1000000)</f>
+        <v/>
+      </c>
+      <c r="U13" s="14">
+        <f>U12/(U11*1000000)</f>
+        <v/>
+      </c>
+      <c r="V13" s="14">
+        <f>V12/(V11*1000000)</f>
+        <v/>
+      </c>
+      <c r="W13" s="14">
+        <f>W12/(W11*1000000)</f>
+        <v/>
+      </c>
+      <c r="X13" s="14">
+        <f>X12/(X11*1000000)</f>
         <v/>
       </c>
     </row>
@@ -1543,6 +1738,11 @@
       <c r="Q14" s="7" t="n"/>
       <c r="R14" s="7" t="n"/>
       <c r="S14" s="7" t="n"/>
+      <c r="T14" s="7" t="n"/>
+      <c r="U14" s="7" t="n"/>
+      <c r="V14" s="7" t="n"/>
+      <c r="W14" s="7" t="n"/>
+      <c r="X14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1610,6 +1810,21 @@
       <c r="S15" s="11" t="n">
         <v>9</v>
       </c>
+      <c r="T15" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="U15" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="V15" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="W15" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="X15" s="11" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1677,6 +1892,21 @@
       <c r="S16" s="11" t="n">
         <v>-0.5</v>
       </c>
+      <c r="T16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="V16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1744,6 +1974,21 @@
       <c r="S17" s="11" t="n">
         <v>0</v>
       </c>
+      <c r="T17" s="11" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="U17" s="11" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="V17" s="11" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="W17" s="11" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="X17" s="11" t="n">
+        <v>-1.5</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1826,6 +2071,26 @@
         <f>S15+S16+S17</f>
         <v/>
       </c>
+      <c r="T18" s="15">
+        <f>T15+T16+T17</f>
+        <v/>
+      </c>
+      <c r="U18" s="15">
+        <f>U15+U16+U17</f>
+        <v/>
+      </c>
+      <c r="V18" s="15">
+        <f>V15+V16+V17</f>
+        <v/>
+      </c>
+      <c r="W18" s="15">
+        <f>W15+W16+W17</f>
+        <v/>
+      </c>
+      <c r="X18" s="15">
+        <f>X15+X16+X17</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1893,6 +2158,21 @@
       <c r="S19" s="16" t="n">
         <v>0</v>
       </c>
+      <c r="T19" s="16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="U19" s="16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="V19" s="16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="W19" s="16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="X19" s="16" t="n">
+        <v>4.5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1975,6 +2255,26 @@
         <f>S18+S19</f>
         <v/>
       </c>
+      <c r="T20" s="15">
+        <f>T18+T19</f>
+        <v/>
+      </c>
+      <c r="U20" s="15">
+        <f>U18+U19</f>
+        <v/>
+      </c>
+      <c r="V20" s="15">
+        <f>V18+V19</f>
+        <v/>
+      </c>
+      <c r="W20" s="15">
+        <f>W18+W19</f>
+        <v/>
+      </c>
+      <c r="X20" s="15">
+        <f>X18+X19</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2055,6 +2355,26 @@
       </c>
       <c r="S21" s="15">
         <f>S20-2.15</f>
+        <v/>
+      </c>
+      <c r="T21" s="15">
+        <f>T20-2.15</f>
+        <v/>
+      </c>
+      <c r="U21" s="15">
+        <f>U20-2.15</f>
+        <v/>
+      </c>
+      <c r="V21" s="15">
+        <f>V20-2.15</f>
+        <v/>
+      </c>
+      <c r="W21" s="15">
+        <f>W20-2.15</f>
+        <v/>
+      </c>
+      <c r="X21" s="15">
+        <f>X20-2.15</f>
         <v/>
       </c>
     </row>
@@ -2129,6 +2449,26 @@
       </c>
       <c r="S22" s="17">
         <f>IF(IF(S8="ERP",S21,S20)&lt;=S9,"OK","OVER LIMIT")</f>
+        <v/>
+      </c>
+      <c r="T22" s="17">
+        <f>IF(IF(T8="ERP",T21,T20)&lt;=T9,"OK","OVER LIMIT")</f>
+        <v/>
+      </c>
+      <c r="U22" s="17">
+        <f>IF(IF(U8="ERP",U21,U20)&lt;=U9,"OK","OVER LIMIT")</f>
+        <v/>
+      </c>
+      <c r="V22" s="17">
+        <f>IF(IF(V8="ERP",V21,V20)&lt;=V9,"OK","OVER LIMIT")</f>
+        <v/>
+      </c>
+      <c r="W22" s="17">
+        <f>IF(IF(W8="ERP",W21,W20)&lt;=W9,"OK","OVER LIMIT")</f>
+        <v/>
+      </c>
+      <c r="X22" s="17">
+        <f>IF(IF(X8="ERP",X21,X20)&lt;=X9,"OK","OVER LIMIT")</f>
         <v/>
       </c>
     </row>
@@ -2156,6 +2496,11 @@
       <c r="Q23" s="7" t="n"/>
       <c r="R23" s="7" t="n"/>
       <c r="S23" s="7" t="n"/>
+      <c r="T23" s="7" t="n"/>
+      <c r="U23" s="7" t="n"/>
+      <c r="V23" s="7" t="n"/>
+      <c r="W23" s="7" t="n"/>
+      <c r="X23" s="7" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2219,6 +2564,21 @@
       <c r="S24" s="13" t="n">
         <v>70</v>
       </c>
+      <c r="T24" s="13" t="n">
+        <v>70</v>
+      </c>
+      <c r="U24" s="13" t="n">
+        <v>70</v>
+      </c>
+      <c r="V24" s="13" t="n">
+        <v>260</v>
+      </c>
+      <c r="W24" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="X24" s="13" t="n">
+        <v>260</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2284,6 +2644,21 @@
         <v>0.75</v>
       </c>
       <c r="S25" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="T25" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="U25" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="V25" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="W25" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="X25" s="18" t="n">
         <v>0.75</v>
       </c>
     </row>
@@ -2349,6 +2724,21 @@
       <c r="S26" s="18" t="n">
         <v>0.75</v>
       </c>
+      <c r="T26" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="U26" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="V26" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="W26" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="X26" s="18" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2416,6 +2806,21 @@
       <c r="S27" s="19" t="n">
         <v>1</v>
       </c>
+      <c r="T27" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="U27" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="V27" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="W27" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="X27" s="19" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2498,6 +2903,26 @@
         <f>SQRT(S24^2+(S25+S26)^2)-SQRT(S24^2+(S25-S26)^2)</f>
         <v/>
       </c>
+      <c r="T28" s="20">
+        <f>SQRT(T24^2+(T25+T26)^2)-SQRT(T24^2+(T25-T26)^2)</f>
+        <v/>
+      </c>
+      <c r="U28" s="20">
+        <f>SQRT(U24^2+(U25+U26)^2)-SQRT(U24^2+(U25-U26)^2)</f>
+        <v/>
+      </c>
+      <c r="V28" s="20">
+        <f>SQRT(V24^2+(V25+V26)^2)-SQRT(V24^2+(V25-V26)^2)</f>
+        <v/>
+      </c>
+      <c r="W28" s="20">
+        <f>SQRT(W24^2+(W25+W26)^2)-SQRT(W24^2+(W25-W26)^2)</f>
+        <v/>
+      </c>
+      <c r="X28" s="20">
+        <f>SQRT(X24^2+(X25+X26)^2)-SQRT(X24^2+(X25-X26)^2)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2578,6 +3003,26 @@
       </c>
       <c r="S29" s="21">
         <f>2*PI()*S28/S13</f>
+        <v/>
+      </c>
+      <c r="T29" s="21">
+        <f>2*PI()*T28/T13</f>
+        <v/>
+      </c>
+      <c r="U29" s="21">
+        <f>2*PI()*U28/U13</f>
+        <v/>
+      </c>
+      <c r="V29" s="21">
+        <f>2*PI()*V28/V13</f>
+        <v/>
+      </c>
+      <c r="W29" s="21">
+        <f>2*PI()*W28/W13</f>
+        <v/>
+      </c>
+      <c r="X29" s="21">
+        <f>2*PI()*X28/X13</f>
         <v/>
       </c>
     </row>
@@ -2654,6 +3099,26 @@
         <f>IF(S29&lt;PI()/2,"beyond breakpoint","interference zone")</f>
         <v/>
       </c>
+      <c r="T30" s="17">
+        <f>IF(T29&lt;PI()/2,"beyond breakpoint","interference zone")</f>
+        <v/>
+      </c>
+      <c r="U30" s="17">
+        <f>IF(U29&lt;PI()/2,"beyond breakpoint","interference zone")</f>
+        <v/>
+      </c>
+      <c r="V30" s="17">
+        <f>IF(V29&lt;PI()/2,"beyond breakpoint","interference zone")</f>
+        <v/>
+      </c>
+      <c r="W30" s="17">
+        <f>IF(W29&lt;PI()/2,"beyond breakpoint","interference zone")</f>
+        <v/>
+      </c>
+      <c r="X30" s="17">
+        <f>IF(X29&lt;PI()/2,"beyond breakpoint","interference zone")</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2736,6 +3201,26 @@
         <f>20*LOG10(S13/(4*PI()*S24))</f>
         <v/>
       </c>
+      <c r="T31" s="15">
+        <f>20*LOG10(T13/(4*PI()*T24))</f>
+        <v/>
+      </c>
+      <c r="U31" s="15">
+        <f>20*LOG10(U13/(4*PI()*U24))</f>
+        <v/>
+      </c>
+      <c r="V31" s="15">
+        <f>20*LOG10(V13/(4*PI()*V24))</f>
+        <v/>
+      </c>
+      <c r="W31" s="15">
+        <f>20*LOG10(W13/(4*PI()*W24))</f>
+        <v/>
+      </c>
+      <c r="X31" s="15">
+        <f>20*LOG10(X13/(4*PI()*X24))</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2818,6 +3303,26 @@
         <f>10*LOG10(1+S27^2-2*S27*ABS(COS(S29)))</f>
         <v/>
       </c>
+      <c r="T32" s="15">
+        <f>10*LOG10(1+T27^2-2*T27*ABS(COS(T29)))</f>
+        <v/>
+      </c>
+      <c r="U32" s="15">
+        <f>10*LOG10(1+U27^2-2*U27*ABS(COS(U29)))</f>
+        <v/>
+      </c>
+      <c r="V32" s="15">
+        <f>10*LOG10(1+V27^2-2*V27*ABS(COS(V29)))</f>
+        <v/>
+      </c>
+      <c r="W32" s="15">
+        <f>10*LOG10(1+W27^2-2*W27*ABS(COS(W29)))</f>
+        <v/>
+      </c>
+      <c r="X32" s="15">
+        <f>10*LOG10(1+X27^2-2*X27*ABS(COS(X29)))</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2900,6 +3405,26 @@
         <f>S31+S32</f>
         <v/>
       </c>
+      <c r="T33" s="15">
+        <f>T31+T32</f>
+        <v/>
+      </c>
+      <c r="U33" s="15">
+        <f>U31+U32</f>
+        <v/>
+      </c>
+      <c r="V33" s="15">
+        <f>V31+V32</f>
+        <v/>
+      </c>
+      <c r="W33" s="15">
+        <f>W31+W32</f>
+        <v/>
+      </c>
+      <c r="X33" s="15">
+        <f>X31+X32</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2967,6 +3492,21 @@
       <c r="S34" s="16" t="n">
         <v>-1</v>
       </c>
+      <c r="T34" s="16" t="n">
+        <v>-1</v>
+      </c>
+      <c r="U34" s="16" t="n">
+        <v>-1</v>
+      </c>
+      <c r="V34" s="16" t="n">
+        <v>-1</v>
+      </c>
+      <c r="W34" s="16" t="n">
+        <v>-1</v>
+      </c>
+      <c r="X34" s="16" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3034,6 +3574,21 @@
       <c r="S35" s="16" t="n">
         <v>0</v>
       </c>
+      <c r="T35" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="U35" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="V35" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="W35" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="X35" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3101,6 +3656,21 @@
       <c r="S36" s="16" t="n">
         <v>0</v>
       </c>
+      <c r="T36" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="U36" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="V36" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="W36" s="16" t="n">
+        <v>-10</v>
+      </c>
+      <c r="X36" s="16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3183,6 +3753,26 @@
         <f>S20+S31+S34</f>
         <v/>
       </c>
+      <c r="T37" s="15">
+        <f>T20+T31+T34</f>
+        <v/>
+      </c>
+      <c r="U37" s="15">
+        <f>U20+U31+U34</f>
+        <v/>
+      </c>
+      <c r="V37" s="15">
+        <f>V20+V31+V34</f>
+        <v/>
+      </c>
+      <c r="W37" s="15">
+        <f>W20+W31+W34</f>
+        <v/>
+      </c>
+      <c r="X37" s="15">
+        <f>X20+X31+X34</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3263,6 +3853,26 @@
       </c>
       <c r="S38" s="15">
         <f>S20+S33+S34+S35+S36</f>
+        <v/>
+      </c>
+      <c r="T38" s="15">
+        <f>T20+T33+T34+T35+T36</f>
+        <v/>
+      </c>
+      <c r="U38" s="15">
+        <f>U20+U33+U34+U35+U36</f>
+        <v/>
+      </c>
+      <c r="V38" s="15">
+        <f>V20+V33+V34+V35+V36</f>
+        <v/>
+      </c>
+      <c r="W38" s="15">
+        <f>W20+W33+W34+W35+W36</f>
+        <v/>
+      </c>
+      <c r="X38" s="15">
+        <f>X20+X33+X34+X35+X36</f>
         <v/>
       </c>
     </row>
@@ -3290,6 +3900,11 @@
       <c r="Q39" s="7" t="n"/>
       <c r="R39" s="7" t="n"/>
       <c r="S39" s="7" t="n"/>
+      <c r="T39" s="7" t="n"/>
+      <c r="U39" s="7" t="n"/>
+      <c r="V39" s="7" t="n"/>
+      <c r="W39" s="7" t="n"/>
+      <c r="X39" s="7" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3357,6 +3972,21 @@
       <c r="S40" s="16" t="n">
         <v>0</v>
       </c>
+      <c r="T40" s="16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="U40" s="16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="V40" s="16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="W40" s="16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="X40" s="16" t="n">
+        <v>4.5</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3420,6 +4050,21 @@
       <c r="S41" s="11" t="n">
         <v>0</v>
       </c>
+      <c r="T41" s="11" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="U41" s="11" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="V41" s="11" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="W41" s="11" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="X41" s="11" t="n">
+        <v>-1.5</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3502,6 +4147,26 @@
         <f>S37+S40+S41</f>
         <v/>
       </c>
+      <c r="T42" s="15">
+        <f>T37+T40+T41</f>
+        <v/>
+      </c>
+      <c r="U42" s="15">
+        <f>U37+U40+U41</f>
+        <v/>
+      </c>
+      <c r="V42" s="15">
+        <f>V37+V40+V41</f>
+        <v/>
+      </c>
+      <c r="W42" s="15">
+        <f>W37+W40+W41</f>
+        <v/>
+      </c>
+      <c r="X42" s="15">
+        <f>X37+X40+X41</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3584,6 +4249,26 @@
         <f>S38+S40+S41</f>
         <v/>
       </c>
+      <c r="T43" s="15">
+        <f>T38+T40+T41</f>
+        <v/>
+      </c>
+      <c r="U43" s="15">
+        <f>U38+U40+U41</f>
+        <v/>
+      </c>
+      <c r="V43" s="15">
+        <f>V38+V40+V41</f>
+        <v/>
+      </c>
+      <c r="W43" s="15">
+        <f>W38+W40+W41</f>
+        <v/>
+      </c>
+      <c r="X43" s="15">
+        <f>X38+X40+X41</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3650,6 +4335,21 @@
       </c>
       <c r="S44" s="9" t="n">
         <v>-100</v>
+      </c>
+      <c r="T44" s="9" t="n">
+        <v>-94</v>
+      </c>
+      <c r="U44" s="9" t="n">
+        <v>-85</v>
+      </c>
+      <c r="V44" s="9" t="n">
+        <v>-94</v>
+      </c>
+      <c r="W44" s="9" t="n">
+        <v>-94</v>
+      </c>
+      <c r="X44" s="9" t="n">
+        <v>-94</v>
       </c>
     </row>
     <row r="45" ht="60" customHeight="1">
@@ -3734,6 +4434,31 @@
       <c r="S45" s="8" t="inlineStr">
         <is>
           <t>ESTIMATE: datasheet stops at 38.4 kbps (-105 dBm); ~-5 dB for 2x bandwidth. Measure on the bench.</t>
+        </is>
+      </c>
+      <c r="T45" s="8" t="inlineStr">
+        <is>
+          <t>nRF24L01+ chip datasheet: -94 dBm @250 kbps; module LNA ignored (Ebyte quotes ~-96 @250k for the sister E01-ML01SP4). Measure in T2.</t>
+        </is>
+      </c>
+      <c r="U45" s="8" t="inlineStr">
+        <is>
+          <t>nRF24L01+ chip datasheet: -85 dBm @1000 kbps; module LNA ignored (Ebyte quotes ~-96 @250k for the sister E01-ML01SP4). Measure in T2.</t>
+        </is>
+      </c>
+      <c r="V45" s="8" t="inlineStr">
+        <is>
+          <t>nRF24L01+ chip datasheet: -94 dBm @250 kbps; module LNA ignored (Ebyte quotes ~-96 @250k for the sister E01-ML01SP4). Measure in T2.</t>
+        </is>
+      </c>
+      <c r="W45" s="8" t="inlineStr">
+        <is>
+          <t>nRF24L01+ chip datasheet: -94 dBm @250 kbps; module LNA ignored (Ebyte quotes ~-96 @250k for the sister E01-ML01SP4). Measure in T2.</t>
+        </is>
+      </c>
+      <c r="X45" s="8" t="inlineStr">
+        <is>
+          <t>nRF24L01+ chip datasheet: -94 dBm @250 kbps; module LNA ignored (Ebyte quotes ~-96 @250k for the sister E01-ML01SP4). Measure in T2.</t>
         </is>
       </c>
     </row>
@@ -3761,6 +4486,11 @@
       <c r="Q46" s="7" t="n"/>
       <c r="R46" s="7" t="n"/>
       <c r="S46" s="7" t="n"/>
+      <c r="T46" s="7" t="n"/>
+      <c r="U46" s="7" t="n"/>
+      <c r="V46" s="7" t="n"/>
+      <c r="W46" s="7" t="n"/>
+      <c r="X46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3843,6 +4573,26 @@
         <f>S42-S44</f>
         <v/>
       </c>
+      <c r="T47" s="22">
+        <f>T42-T44</f>
+        <v/>
+      </c>
+      <c r="U47" s="22">
+        <f>U42-U44</f>
+        <v/>
+      </c>
+      <c r="V47" s="22">
+        <f>V42-V44</f>
+        <v/>
+      </c>
+      <c r="W47" s="22">
+        <f>W42-W44</f>
+        <v/>
+      </c>
+      <c r="X47" s="22">
+        <f>X42-X44</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -3925,6 +4675,26 @@
         <f>S43-S44</f>
         <v/>
       </c>
+      <c r="T48" s="23">
+        <f>T43-T44</f>
+        <v/>
+      </c>
+      <c r="U48" s="23">
+        <f>U43-U44</f>
+        <v/>
+      </c>
+      <c r="V48" s="23">
+        <f>V43-V44</f>
+        <v/>
+      </c>
+      <c r="W48" s="23">
+        <f>W43-W44</f>
+        <v/>
+      </c>
+      <c r="X48" s="23">
+        <f>X43-X44</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3999,6 +4769,26 @@
       </c>
       <c r="S49" s="22">
         <f>S43-S35+$D$49-S44</f>
+        <v/>
+      </c>
+      <c r="T49" s="22">
+        <f>T43-T35+$D$49-T44</f>
+        <v/>
+      </c>
+      <c r="U49" s="22">
+        <f>U43-U35+$D$49-U44</f>
+        <v/>
+      </c>
+      <c r="V49" s="22">
+        <f>V43-V35+$D$49-V44</f>
+        <v/>
+      </c>
+      <c r="W49" s="22">
+        <f>W43-W35+$D$49-W44</f>
+        <v/>
+      </c>
+      <c r="X49" s="22">
+        <f>X43-X35+$D$49-X44</f>
         <v/>
       </c>
     </row>
@@ -4026,6 +4816,11 @@
       <c r="Q50" s="7" t="n"/>
       <c r="R50" s="7" t="n"/>
       <c r="S50" s="7" t="n"/>
+      <c r="T50" s="7" t="n"/>
+      <c r="U50" s="7" t="n"/>
+      <c r="V50" s="7" t="n"/>
+      <c r="W50" s="7" t="n"/>
+      <c r="X50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4092,6 +4887,21 @@
       </c>
       <c r="S51" s="11" t="n">
         <v>7</v>
+      </c>
+      <c r="T51" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="U51" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="V51" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="W51" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="X51" s="11" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="52">
@@ -4156,6 +4966,21 @@
       <c r="S52" s="13" t="n">
         <v>290</v>
       </c>
+      <c r="T52" s="13" t="n">
+        <v>290</v>
+      </c>
+      <c r="U52" s="13" t="n">
+        <v>290</v>
+      </c>
+      <c r="V52" s="13" t="n">
+        <v>290</v>
+      </c>
+      <c r="W52" s="13" t="n">
+        <v>290</v>
+      </c>
+      <c r="X52" s="13" t="n">
+        <v>290</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4238,6 +5063,26 @@
         <f>S52*(10^(S51/10)-1)</f>
         <v/>
       </c>
+      <c r="T53" s="25">
+        <f>T52*(10^(T51/10)-1)</f>
+        <v/>
+      </c>
+      <c r="U53" s="25">
+        <f>U52*(10^(U51/10)-1)</f>
+        <v/>
+      </c>
+      <c r="V53" s="25">
+        <f>V52*(10^(V51/10)-1)</f>
+        <v/>
+      </c>
+      <c r="W53" s="25">
+        <f>W52*(10^(W51/10)-1)</f>
+        <v/>
+      </c>
+      <c r="X53" s="25">
+        <f>X52*(10^(X51/10)-1)</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4304,6 +5149,21 @@
       </c>
       <c r="S54" s="13" t="n">
         <v>200</v>
+      </c>
+      <c r="T54" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="U54" s="13" t="n">
+        <v>1000</v>
+      </c>
+      <c r="V54" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="W54" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="X54" s="13" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="55">
@@ -4368,6 +5228,21 @@
       <c r="S55" s="13" t="n">
         <v>300</v>
       </c>
+      <c r="T55" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="U55" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="V55" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="W55" s="13" t="n">
+        <v>300</v>
+      </c>
+      <c r="X55" s="13" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4435,6 +5310,21 @@
       <c r="S56" s="19" t="n">
         <v>1.38</v>
       </c>
+      <c r="T56" s="19" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="U56" s="19" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="V56" s="19" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="W56" s="19" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="X56" s="19" t="n">
+        <v>1.38</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4517,6 +5407,26 @@
         <f>10*LOG10(S56*(S55+S53)*S54*1000)-230+30</f>
         <v/>
       </c>
+      <c r="T57" s="15">
+        <f>10*LOG10(T56*(T55+T53)*T54*1000)-230+30</f>
+        <v/>
+      </c>
+      <c r="U57" s="15">
+        <f>10*LOG10(U56*(U55+U53)*U54*1000)-230+30</f>
+        <v/>
+      </c>
+      <c r="V57" s="15">
+        <f>10*LOG10(V56*(V55+V53)*V54*1000)-230+30</f>
+        <v/>
+      </c>
+      <c r="W57" s="15">
+        <f>10*LOG10(W56*(W55+W53)*W54*1000)-230+30</f>
+        <v/>
+      </c>
+      <c r="X57" s="15">
+        <f>10*LOG10(X56*(X55+X53)*X54*1000)-230+30</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4595,6 +5505,26 @@
         <f>S44-S57</f>
         <v/>
       </c>
+      <c r="T58" s="15">
+        <f>T44-T57</f>
+        <v/>
+      </c>
+      <c r="U58" s="15">
+        <f>U44-U57</f>
+        <v/>
+      </c>
+      <c r="V58" s="15">
+        <f>V44-V57</f>
+        <v/>
+      </c>
+      <c r="W58" s="15">
+        <f>W44-W57</f>
+        <v/>
+      </c>
+      <c r="X58" s="15">
+        <f>X44-X57</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4677,6 +5607,26 @@
         <f>S43-S57</f>
         <v/>
       </c>
+      <c r="T59" s="15">
+        <f>T43-T57</f>
+        <v/>
+      </c>
+      <c r="U59" s="15">
+        <f>U43-U57</f>
+        <v/>
+      </c>
+      <c r="V59" s="15">
+        <f>V43-V57</f>
+        <v/>
+      </c>
+      <c r="W59" s="15">
+        <f>W43-W57</f>
+        <v/>
+      </c>
+      <c r="X59" s="15">
+        <f>X43-X57</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -4862,6 +5812,66 @@
       <c r="D76" s="4" t="inlineStr">
         <is>
           <t>869.70-870.00 MHz: 5 mW e.r.p., no duty-cycle limit; for repeated tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>S16: SRI 70 m | E01-ML01DP5 2.4G | 250 kbps, patches (2.4 baseline)</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>E01-ML01DP5 @RF_PWR -18 (~+7 dBm, est.), 1 dB pigtail + 0.5 dB pad, 4.5 dBi FR4 patch</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>S17: SRI 70 m | E01-ML01DP5 2.4G | 1 Mbps, patches</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>E01-ML01DP5 @RF_PWR -18 (~+7 dBm, est.), 1 dB pigtail + 0.5 dB pad, 4.5 dBi FR4 patch</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>S18: MRM 260 m | E01-ML01DP5 2.4G | 250 kbps, patches (2.4 baseline)</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>E01-ML01DP5 @RF_PWR -18 (~+7 dBm, est.), 1 dB pigtail + 0.5 dB pad, 4.5 dBi FR4 patch</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>S19: NM hop 100 m | E01-ML01DP5 2.4G | 250 kbps, -10 dB obstr. (2.4 baseline)</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>E01-ML01DP5 @RF_PWR -18 (~+7 dBm, est.), 1 dB pigtail + 0.5 dB pad, 4.5 dBi FR4 patch</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>S20: MRM 260 m | E01-ML01DP5 2.4G | 250 kbps, 100 mW FHSS (if Atenea Q3 = yes)</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>UN-85 a) FHSS: 100 mW e.i.r.p.; needs &gt;=15 hop channels + EN 300 328 adaptivity</t>
         </is>
       </c>
     </row>
@@ -4880,7 +5890,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -5314,6 +6324,136 @@
       </c>
       <c r="F19" s="28">
         <f>'Link Budget'!S20+20*LOG10('Link Budget'!S13/(4*PI()*'Link Budget'!S24))+10*LOG10(1+'Link Budget'!S27^2-2*'Link Budget'!S27*ABS(COS(2*PI()*(SQRT('Link Budget'!S24^2+(2*F$4)^2)-'Link Budget'!S24)/'Link Budget'!S13)))+'Link Budget'!S34+'Link Budget'!S35+'Link Budget'!S36+'Link Budget'!S40+'Link Budget'!S41-'Link Budget'!S44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="27">
+        <f>"S16  "&amp;'Link Budget'!T5&amp;" | "&amp;'Link Budget'!T6</f>
+        <v/>
+      </c>
+      <c r="B20" s="28">
+        <f>'Link Budget'!T20+20*LOG10('Link Budget'!T13/(4*PI()*'Link Budget'!T24))+10*LOG10(1+'Link Budget'!T27^2-2*'Link Budget'!T27*ABS(COS(2*PI()*(SQRT('Link Budget'!T24^2+(2*B$4)^2)-'Link Budget'!T24)/'Link Budget'!T13)))+'Link Budget'!T34+'Link Budget'!T35+'Link Budget'!T36+'Link Budget'!T40+'Link Budget'!T41-'Link Budget'!T44</f>
+        <v/>
+      </c>
+      <c r="C20" s="28">
+        <f>'Link Budget'!T20+20*LOG10('Link Budget'!T13/(4*PI()*'Link Budget'!T24))+10*LOG10(1+'Link Budget'!T27^2-2*'Link Budget'!T27*ABS(COS(2*PI()*(SQRT('Link Budget'!T24^2+(2*C$4)^2)-'Link Budget'!T24)/'Link Budget'!T13)))+'Link Budget'!T34+'Link Budget'!T35+'Link Budget'!T36+'Link Budget'!T40+'Link Budget'!T41-'Link Budget'!T44</f>
+        <v/>
+      </c>
+      <c r="D20" s="28">
+        <f>'Link Budget'!T20+20*LOG10('Link Budget'!T13/(4*PI()*'Link Budget'!T24))+10*LOG10(1+'Link Budget'!T27^2-2*'Link Budget'!T27*ABS(COS(2*PI()*(SQRT('Link Budget'!T24^2+(2*D$4)^2)-'Link Budget'!T24)/'Link Budget'!T13)))+'Link Budget'!T34+'Link Budget'!T35+'Link Budget'!T36+'Link Budget'!T40+'Link Budget'!T41-'Link Budget'!T44</f>
+        <v/>
+      </c>
+      <c r="E20" s="28">
+        <f>'Link Budget'!T20+20*LOG10('Link Budget'!T13/(4*PI()*'Link Budget'!T24))+10*LOG10(1+'Link Budget'!T27^2-2*'Link Budget'!T27*ABS(COS(2*PI()*(SQRT('Link Budget'!T24^2+(2*E$4)^2)-'Link Budget'!T24)/'Link Budget'!T13)))+'Link Budget'!T34+'Link Budget'!T35+'Link Budget'!T36+'Link Budget'!T40+'Link Budget'!T41-'Link Budget'!T44</f>
+        <v/>
+      </c>
+      <c r="F20" s="28">
+        <f>'Link Budget'!T20+20*LOG10('Link Budget'!T13/(4*PI()*'Link Budget'!T24))+10*LOG10(1+'Link Budget'!T27^2-2*'Link Budget'!T27*ABS(COS(2*PI()*(SQRT('Link Budget'!T24^2+(2*F$4)^2)-'Link Budget'!T24)/'Link Budget'!T13)))+'Link Budget'!T34+'Link Budget'!T35+'Link Budget'!T36+'Link Budget'!T40+'Link Budget'!T41-'Link Budget'!T44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="27">
+        <f>"S17  "&amp;'Link Budget'!U5&amp;" | "&amp;'Link Budget'!U6</f>
+        <v/>
+      </c>
+      <c r="B21" s="28">
+        <f>'Link Budget'!U20+20*LOG10('Link Budget'!U13/(4*PI()*'Link Budget'!U24))+10*LOG10(1+'Link Budget'!U27^2-2*'Link Budget'!U27*ABS(COS(2*PI()*(SQRT('Link Budget'!U24^2+(2*B$4)^2)-'Link Budget'!U24)/'Link Budget'!U13)))+'Link Budget'!U34+'Link Budget'!U35+'Link Budget'!U36+'Link Budget'!U40+'Link Budget'!U41-'Link Budget'!U44</f>
+        <v/>
+      </c>
+      <c r="C21" s="28">
+        <f>'Link Budget'!U20+20*LOG10('Link Budget'!U13/(4*PI()*'Link Budget'!U24))+10*LOG10(1+'Link Budget'!U27^2-2*'Link Budget'!U27*ABS(COS(2*PI()*(SQRT('Link Budget'!U24^2+(2*C$4)^2)-'Link Budget'!U24)/'Link Budget'!U13)))+'Link Budget'!U34+'Link Budget'!U35+'Link Budget'!U36+'Link Budget'!U40+'Link Budget'!U41-'Link Budget'!U44</f>
+        <v/>
+      </c>
+      <c r="D21" s="28">
+        <f>'Link Budget'!U20+20*LOG10('Link Budget'!U13/(4*PI()*'Link Budget'!U24))+10*LOG10(1+'Link Budget'!U27^2-2*'Link Budget'!U27*ABS(COS(2*PI()*(SQRT('Link Budget'!U24^2+(2*D$4)^2)-'Link Budget'!U24)/'Link Budget'!U13)))+'Link Budget'!U34+'Link Budget'!U35+'Link Budget'!U36+'Link Budget'!U40+'Link Budget'!U41-'Link Budget'!U44</f>
+        <v/>
+      </c>
+      <c r="E21" s="28">
+        <f>'Link Budget'!U20+20*LOG10('Link Budget'!U13/(4*PI()*'Link Budget'!U24))+10*LOG10(1+'Link Budget'!U27^2-2*'Link Budget'!U27*ABS(COS(2*PI()*(SQRT('Link Budget'!U24^2+(2*E$4)^2)-'Link Budget'!U24)/'Link Budget'!U13)))+'Link Budget'!U34+'Link Budget'!U35+'Link Budget'!U36+'Link Budget'!U40+'Link Budget'!U41-'Link Budget'!U44</f>
+        <v/>
+      </c>
+      <c r="F21" s="28">
+        <f>'Link Budget'!U20+20*LOG10('Link Budget'!U13/(4*PI()*'Link Budget'!U24))+10*LOG10(1+'Link Budget'!U27^2-2*'Link Budget'!U27*ABS(COS(2*PI()*(SQRT('Link Budget'!U24^2+(2*F$4)^2)-'Link Budget'!U24)/'Link Budget'!U13)))+'Link Budget'!U34+'Link Budget'!U35+'Link Budget'!U36+'Link Budget'!U40+'Link Budget'!U41-'Link Budget'!U44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="27">
+        <f>"S18  "&amp;'Link Budget'!V5&amp;" | "&amp;'Link Budget'!V6</f>
+        <v/>
+      </c>
+      <c r="B22" s="28">
+        <f>'Link Budget'!V20+20*LOG10('Link Budget'!V13/(4*PI()*'Link Budget'!V24))+10*LOG10(1+'Link Budget'!V27^2-2*'Link Budget'!V27*ABS(COS(2*PI()*(SQRT('Link Budget'!V24^2+(2*B$4)^2)-'Link Budget'!V24)/'Link Budget'!V13)))+'Link Budget'!V34+'Link Budget'!V35+'Link Budget'!V36+'Link Budget'!V40+'Link Budget'!V41-'Link Budget'!V44</f>
+        <v/>
+      </c>
+      <c r="C22" s="28">
+        <f>'Link Budget'!V20+20*LOG10('Link Budget'!V13/(4*PI()*'Link Budget'!V24))+10*LOG10(1+'Link Budget'!V27^2-2*'Link Budget'!V27*ABS(COS(2*PI()*(SQRT('Link Budget'!V24^2+(2*C$4)^2)-'Link Budget'!V24)/'Link Budget'!V13)))+'Link Budget'!V34+'Link Budget'!V35+'Link Budget'!V36+'Link Budget'!V40+'Link Budget'!V41-'Link Budget'!V44</f>
+        <v/>
+      </c>
+      <c r="D22" s="28">
+        <f>'Link Budget'!V20+20*LOG10('Link Budget'!V13/(4*PI()*'Link Budget'!V24))+10*LOG10(1+'Link Budget'!V27^2-2*'Link Budget'!V27*ABS(COS(2*PI()*(SQRT('Link Budget'!V24^2+(2*D$4)^2)-'Link Budget'!V24)/'Link Budget'!V13)))+'Link Budget'!V34+'Link Budget'!V35+'Link Budget'!V36+'Link Budget'!V40+'Link Budget'!V41-'Link Budget'!V44</f>
+        <v/>
+      </c>
+      <c r="E22" s="28">
+        <f>'Link Budget'!V20+20*LOG10('Link Budget'!V13/(4*PI()*'Link Budget'!V24))+10*LOG10(1+'Link Budget'!V27^2-2*'Link Budget'!V27*ABS(COS(2*PI()*(SQRT('Link Budget'!V24^2+(2*E$4)^2)-'Link Budget'!V24)/'Link Budget'!V13)))+'Link Budget'!V34+'Link Budget'!V35+'Link Budget'!V36+'Link Budget'!V40+'Link Budget'!V41-'Link Budget'!V44</f>
+        <v/>
+      </c>
+      <c r="F22" s="28">
+        <f>'Link Budget'!V20+20*LOG10('Link Budget'!V13/(4*PI()*'Link Budget'!V24))+10*LOG10(1+'Link Budget'!V27^2-2*'Link Budget'!V27*ABS(COS(2*PI()*(SQRT('Link Budget'!V24^2+(2*F$4)^2)-'Link Budget'!V24)/'Link Budget'!V13)))+'Link Budget'!V34+'Link Budget'!V35+'Link Budget'!V36+'Link Budget'!V40+'Link Budget'!V41-'Link Budget'!V44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="27">
+        <f>"S19  "&amp;'Link Budget'!W5&amp;" | "&amp;'Link Budget'!W6</f>
+        <v/>
+      </c>
+      <c r="B23" s="28">
+        <f>'Link Budget'!W20+20*LOG10('Link Budget'!W13/(4*PI()*'Link Budget'!W24))+10*LOG10(1+'Link Budget'!W27^2-2*'Link Budget'!W27*ABS(COS(2*PI()*(SQRT('Link Budget'!W24^2+(2*B$4)^2)-'Link Budget'!W24)/'Link Budget'!W13)))+'Link Budget'!W34+'Link Budget'!W35+'Link Budget'!W36+'Link Budget'!W40+'Link Budget'!W41-'Link Budget'!W44</f>
+        <v/>
+      </c>
+      <c r="C23" s="28">
+        <f>'Link Budget'!W20+20*LOG10('Link Budget'!W13/(4*PI()*'Link Budget'!W24))+10*LOG10(1+'Link Budget'!W27^2-2*'Link Budget'!W27*ABS(COS(2*PI()*(SQRT('Link Budget'!W24^2+(2*C$4)^2)-'Link Budget'!W24)/'Link Budget'!W13)))+'Link Budget'!W34+'Link Budget'!W35+'Link Budget'!W36+'Link Budget'!W40+'Link Budget'!W41-'Link Budget'!W44</f>
+        <v/>
+      </c>
+      <c r="D23" s="28">
+        <f>'Link Budget'!W20+20*LOG10('Link Budget'!W13/(4*PI()*'Link Budget'!W24))+10*LOG10(1+'Link Budget'!W27^2-2*'Link Budget'!W27*ABS(COS(2*PI()*(SQRT('Link Budget'!W24^2+(2*D$4)^2)-'Link Budget'!W24)/'Link Budget'!W13)))+'Link Budget'!W34+'Link Budget'!W35+'Link Budget'!W36+'Link Budget'!W40+'Link Budget'!W41-'Link Budget'!W44</f>
+        <v/>
+      </c>
+      <c r="E23" s="28">
+        <f>'Link Budget'!W20+20*LOG10('Link Budget'!W13/(4*PI()*'Link Budget'!W24))+10*LOG10(1+'Link Budget'!W27^2-2*'Link Budget'!W27*ABS(COS(2*PI()*(SQRT('Link Budget'!W24^2+(2*E$4)^2)-'Link Budget'!W24)/'Link Budget'!W13)))+'Link Budget'!W34+'Link Budget'!W35+'Link Budget'!W36+'Link Budget'!W40+'Link Budget'!W41-'Link Budget'!W44</f>
+        <v/>
+      </c>
+      <c r="F23" s="28">
+        <f>'Link Budget'!W20+20*LOG10('Link Budget'!W13/(4*PI()*'Link Budget'!W24))+10*LOG10(1+'Link Budget'!W27^2-2*'Link Budget'!W27*ABS(COS(2*PI()*(SQRT('Link Budget'!W24^2+(2*F$4)^2)-'Link Budget'!W24)/'Link Budget'!W13)))+'Link Budget'!W34+'Link Budget'!W35+'Link Budget'!W36+'Link Budget'!W40+'Link Budget'!W41-'Link Budget'!W44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="27">
+        <f>"S20  "&amp;'Link Budget'!X5&amp;" | "&amp;'Link Budget'!X6</f>
+        <v/>
+      </c>
+      <c r="B24" s="28">
+        <f>'Link Budget'!X20+20*LOG10('Link Budget'!X13/(4*PI()*'Link Budget'!X24))+10*LOG10(1+'Link Budget'!X27^2-2*'Link Budget'!X27*ABS(COS(2*PI()*(SQRT('Link Budget'!X24^2+(2*B$4)^2)-'Link Budget'!X24)/'Link Budget'!X13)))+'Link Budget'!X34+'Link Budget'!X35+'Link Budget'!X36+'Link Budget'!X40+'Link Budget'!X41-'Link Budget'!X44</f>
+        <v/>
+      </c>
+      <c r="C24" s="28">
+        <f>'Link Budget'!X20+20*LOG10('Link Budget'!X13/(4*PI()*'Link Budget'!X24))+10*LOG10(1+'Link Budget'!X27^2-2*'Link Budget'!X27*ABS(COS(2*PI()*(SQRT('Link Budget'!X24^2+(2*C$4)^2)-'Link Budget'!X24)/'Link Budget'!X13)))+'Link Budget'!X34+'Link Budget'!X35+'Link Budget'!X36+'Link Budget'!X40+'Link Budget'!X41-'Link Budget'!X44</f>
+        <v/>
+      </c>
+      <c r="D24" s="28">
+        <f>'Link Budget'!X20+20*LOG10('Link Budget'!X13/(4*PI()*'Link Budget'!X24))+10*LOG10(1+'Link Budget'!X27^2-2*'Link Budget'!X27*ABS(COS(2*PI()*(SQRT('Link Budget'!X24^2+(2*D$4)^2)-'Link Budget'!X24)/'Link Budget'!X13)))+'Link Budget'!X34+'Link Budget'!X35+'Link Budget'!X36+'Link Budget'!X40+'Link Budget'!X41-'Link Budget'!X44</f>
+        <v/>
+      </c>
+      <c r="E24" s="28">
+        <f>'Link Budget'!X20+20*LOG10('Link Budget'!X13/(4*PI()*'Link Budget'!X24))+10*LOG10(1+'Link Budget'!X27^2-2*'Link Budget'!X27*ABS(COS(2*PI()*(SQRT('Link Budget'!X24^2+(2*E$4)^2)-'Link Budget'!X24)/'Link Budget'!X13)))+'Link Budget'!X34+'Link Budget'!X35+'Link Budget'!X36+'Link Budget'!X40+'Link Budget'!X41-'Link Budget'!X44</f>
+        <v/>
+      </c>
+      <c r="F24" s="28">
+        <f>'Link Budget'!X20+20*LOG10('Link Budget'!X13/(4*PI()*'Link Budget'!X24))+10*LOG10(1+'Link Budget'!X27^2-2*'Link Budget'!X27*ABS(COS(2*PI()*(SQRT('Link Budget'!X24^2+(2*F$4)^2)-'Link Budget'!X24)/'Link Budget'!X13)))+'Link Budget'!X34+'Link Budget'!X35+'Link Budget'!X36+'Link Budget'!X40+'Link Budget'!X41-'Link Budget'!X44</f>
         <v/>
       </c>
     </row>
@@ -6017,7 +7157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6354,158 +7494,316 @@
     <row r="8" ht="95" customHeight="1">
       <c r="A8" s="38" t="inlineStr">
         <is>
-          <t>TI CC2500</t>
+          <t>PICK 9-Oct-26: Ebyte E01-ML01DP5 (genuine nRF24L01P + PA/LNA, SMA-K, DIP 2.54 mm)</t>
         </is>
       </c>
       <c r="B8" s="38" t="inlineStr">
         <is>
-          <t>2.400-2.4835 GHz</t>
+          <t>2.400-2.525 GHz (use &lt;=2483.5)</t>
         </is>
       </c>
       <c r="C8" s="38" t="inlineStr">
         <is>
-          <t>+1 dBm</t>
+          <t>+20 dBm; ~+7 dBm at RF_PWR -18 (ESTIMATE, PA ~25 dB gain, no bypass)</t>
         </is>
       </c>
       <c r="D8" s="38" t="inlineStr">
         <is>
-          <t>21.5 mA @+1 dBm</t>
+          <t>~120 mA (sister SP4)</t>
         </is>
       </c>
       <c r="E8" s="38" t="inlineStr">
         <is>
-          <t>~13-17 mA</t>
+          <t>~26 mA (sister SP4)</t>
         </is>
       </c>
       <c r="F8" s="38" t="inlineStr">
         <is>
-          <t>-104 dBm @2.4 kBaud; -99 @10 kBaud; -89 @250 kBaud; -83 @500 kBaud</t>
+          <t>chip -94 dBm @250k / -85 @1M; Ebyte ~-96 @250k for the SP4 (LNA 12 dB, NF 2.5 dB)</t>
         </is>
       </c>
       <c r="G8" s="38" t="inlineStr">
         <is>
-          <t>500 kBaud</t>
+          <t>2 Mbps</t>
         </is>
       </c>
       <c r="H8" s="38" t="inlineStr">
         <is>
-          <t>Similar class to nRF24 with more modulation control.</t>
+          <t>Lowest setting ~+7 dBm: with a 4.5 dBi patch needs ~0.5-3 dB pad for 10 dBm e.i.r.p.; measure (T0). PA/LNA switched inside the module: MCU needs SPI + CE + CSN + IRQ only. 32 B payload.</t>
         </is>
       </c>
       <c r="I8" s="38" t="inlineStr">
         <is>
-          <t>Proprietary - LOW risk</t>
+          <t>Proprietary (Enhanced ShockBurst) - LOW-MEDIUM risk; confirm on Atenea</t>
         </is>
       </c>
       <c r="J8" s="38" t="inlineStr">
         <is>
-          <t>Alternative 2.4 GHz option</t>
+          <t>2.4 GHz baseline, all modes</t>
         </is>
       </c>
       <c r="K8" s="38" t="inlineStr">
         <is>
-          <t>TO VERIFY</t>
+          <t>~US$3.9 (Tindie, EBYTE store) - VERIFY lead time to Spain</t>
         </is>
       </c>
       <c r="L8" s="38" t="inlineStr">
         <is>
-          <t>TI CC2500 datasheet, RF receive section - https://www.ti.com/lit/ds/symlink/cc2500.pdf</t>
+          <t>https://www.cdebyte.com/products/E01-ML01DP5 ; https://voltiq.ru/datasheets/ebyte/E01-ML01SP4.pdf</t>
         </is>
       </c>
     </row>
     <row r="9" ht="95" customHeight="1">
       <c r="A9" s="38" t="inlineStr">
         <is>
-          <t>EXCLUDE: LoRa chips (SX127x/RFM95, SX126x, SX1280, LLCC68)</t>
+          <t>BACKUP: Ebyte E01-ML01SP4 (same radio, SMD 14.85 x 18 mm, IPEX/u.FL)</t>
         </is>
       </c>
       <c r="B9" s="38" t="inlineStr">
         <is>
-          <t>433/868/2.4 GHz</t>
-        </is>
-      </c>
-      <c r="C9" s="38" t="inlineStr"/>
-      <c r="D9" s="38" t="inlineStr"/>
-      <c r="E9" s="38" t="inlineStr"/>
-      <c r="F9" s="38" t="inlineStr"/>
-      <c r="G9" s="38" t="inlineStr"/>
-      <c r="H9" s="38" t="inlineStr"/>
+          <t>2.4 GHz</t>
+        </is>
+      </c>
+      <c r="C9" s="38" t="inlineStr">
+        <is>
+          <t>+20 dBm</t>
+        </is>
+      </c>
+      <c r="D9" s="38" t="inlineStr">
+        <is>
+          <t>120 mA</t>
+        </is>
+      </c>
+      <c r="E9" s="38" t="inlineStr">
+        <is>
+          <t>26 mA</t>
+        </is>
+      </c>
+      <c r="F9" s="38" t="inlineStr">
+        <is>
+          <t>-96 dBm typ @250k (datasheet)</t>
+        </is>
+      </c>
+      <c r="G9" s="38" t="inlineStr">
+        <is>
+          <t>2 Mbps</t>
+        </is>
+      </c>
+      <c r="H9" s="38" t="inlineStr">
+        <is>
+          <t>1.27 mm pitch SMD: solder to the carrier PCB; u.FL to the patch.</t>
+        </is>
+      </c>
       <c r="I9" s="38" t="inlineStr">
         <is>
-          <t>LoRa is named as banned on the Session 1 spec slide; even FSK-only use of a LoRa chip is a compliance risk</t>
+          <t>As above</t>
         </is>
       </c>
       <c r="J9" s="38" t="inlineStr">
         <is>
-          <t>Do not buy</t>
-        </is>
-      </c>
-      <c r="K9" s="38" t="inlineStr"/>
+          <t>Carrier-PCB option</t>
+        </is>
+      </c>
+      <c r="K9" s="38" t="inlineStr">
+        <is>
+          <t>VERIFY</t>
+        </is>
+      </c>
       <c r="L9" s="38" t="inlineStr">
         <is>
-          <t>Session #1 slide 'Transceiver Specs (I)'</t>
+          <t>https://voltiq.ru/datasheets/ebyte/E01-ML01SP4.pdf</t>
         </is>
       </c>
     </row>
     <row r="10" ht="95" customHeight="1">
       <c r="A10" s="38" t="inlineStr">
         <is>
-          <t>EXCLUDE: radio SoCs (CC1310/CC1312, nRF52, ESP32, STM32WL...)</t>
-        </is>
-      </c>
-      <c r="B10" s="38" t="inlineStr"/>
+          <t>EXCLUDE: Ebyte E01C-* and no-name 'nRF24L01+PA+LNA' boards</t>
+        </is>
+      </c>
+      <c r="B10" s="38" t="inlineStr">
+        <is>
+          <t>2.4 GHz</t>
+        </is>
+      </c>
       <c r="C10" s="38" t="inlineStr"/>
       <c r="D10" s="38" t="inlineStr"/>
       <c r="E10" s="38" t="inlineStr"/>
       <c r="F10" s="38" t="inlineStr"/>
       <c r="G10" s="38" t="inlineStr"/>
-      <c r="H10" s="38" t="inlineStr"/>
-      <c r="I10" s="38" t="inlineStr">
-        <is>
-          <t>Contain a microprocessor (second micro module) and/or BLE/ZigBee/LoRa stacks</t>
-        </is>
-      </c>
+      <c r="H10" s="38" t="inlineStr">
+        <is>
+          <t>Ebyte's own E01C manual states the chip is a Si24R1 clone (worse receiver, selectivity unknown)</t>
+        </is>
+      </c>
+      <c r="I10" s="38" t="inlineStr"/>
       <c r="J10" s="38" t="inlineStr">
         <is>
-          <t>Do not buy</t>
+          <t>Do not buy (bench only)</t>
         </is>
       </c>
       <c r="K10" s="38" t="inlineStr"/>
       <c r="L10" s="38" t="inlineStr">
         <is>
-          <t>Rules PDF: 'one but only one module including a microprocessor'; standard-protocol ban</t>
+          <t>https://atta.szlcsc.com/upload/public/pdf/source/20220121/F2AB78B6B3F0E91D6E5268DDE53AA4EA.pdf</t>
         </is>
       </c>
     </row>
     <row r="11" ht="95" customHeight="1">
       <c r="A11" s="38" t="inlineStr">
         <is>
+          <t>TI CC2500</t>
+        </is>
+      </c>
+      <c r="B11" s="38" t="inlineStr">
+        <is>
+          <t>2.400-2.4835 GHz</t>
+        </is>
+      </c>
+      <c r="C11" s="38" t="inlineStr">
+        <is>
+          <t>+1 dBm</t>
+        </is>
+      </c>
+      <c r="D11" s="38" t="inlineStr">
+        <is>
+          <t>21.5 mA @+1 dBm</t>
+        </is>
+      </c>
+      <c r="E11" s="38" t="inlineStr">
+        <is>
+          <t>~13-17 mA</t>
+        </is>
+      </c>
+      <c r="F11" s="38" t="inlineStr">
+        <is>
+          <t>-104 dBm @2.4 kBaud; -99 @10 kBaud; -89 @250 kBaud; -83 @500 kBaud</t>
+        </is>
+      </c>
+      <c r="G11" s="38" t="inlineStr">
+        <is>
+          <t>500 kBaud</t>
+        </is>
+      </c>
+      <c r="H11" s="38" t="inlineStr">
+        <is>
+          <t>Similar class to nRF24 with more modulation control.</t>
+        </is>
+      </c>
+      <c r="I11" s="38" t="inlineStr">
+        <is>
+          <t>Proprietary - LOW risk</t>
+        </is>
+      </c>
+      <c r="J11" s="38" t="inlineStr">
+        <is>
+          <t>Alternative 2.4 GHz option</t>
+        </is>
+      </c>
+      <c r="K11" s="38" t="inlineStr">
+        <is>
+          <t>TO VERIFY</t>
+        </is>
+      </c>
+      <c r="L11" s="38" t="inlineStr">
+        <is>
+          <t>TI CC2500 datasheet, RF receive section - https://www.ti.com/lit/ds/symlink/cc2500.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="95" customHeight="1">
+      <c r="A12" s="38" t="inlineStr">
+        <is>
+          <t>EXCLUDE: LoRa chips (SX127x/RFM95, SX126x, SX1280, LLCC68)</t>
+        </is>
+      </c>
+      <c r="B12" s="38" t="inlineStr">
+        <is>
+          <t>433/868/2.4 GHz</t>
+        </is>
+      </c>
+      <c r="C12" s="38" t="inlineStr"/>
+      <c r="D12" s="38" t="inlineStr"/>
+      <c r="E12" s="38" t="inlineStr"/>
+      <c r="F12" s="38" t="inlineStr"/>
+      <c r="G12" s="38" t="inlineStr"/>
+      <c r="H12" s="38" t="inlineStr"/>
+      <c r="I12" s="38" t="inlineStr">
+        <is>
+          <t>LoRa is named as banned on the Session 1 spec slide; even FSK-only use of a LoRa chip is a compliance risk</t>
+        </is>
+      </c>
+      <c r="J12" s="38" t="inlineStr">
+        <is>
+          <t>Do not buy</t>
+        </is>
+      </c>
+      <c r="K12" s="38" t="inlineStr"/>
+      <c r="L12" s="38" t="inlineStr">
+        <is>
+          <t>Session #1 slide 'Transceiver Specs (I)'</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="95" customHeight="1">
+      <c r="A13" s="38" t="inlineStr">
+        <is>
+          <t>EXCLUDE: radio SoCs (CC1310/CC1312, nRF52, ESP32, STM32WL...)</t>
+        </is>
+      </c>
+      <c r="B13" s="38" t="inlineStr"/>
+      <c r="C13" s="38" t="inlineStr"/>
+      <c r="D13" s="38" t="inlineStr"/>
+      <c r="E13" s="38" t="inlineStr"/>
+      <c r="F13" s="38" t="inlineStr"/>
+      <c r="G13" s="38" t="inlineStr"/>
+      <c r="H13" s="38" t="inlineStr"/>
+      <c r="I13" s="38" t="inlineStr">
+        <is>
+          <t>Contain a microprocessor (second micro module) and/or BLE/ZigBee/LoRa stacks</t>
+        </is>
+      </c>
+      <c r="J13" s="38" t="inlineStr">
+        <is>
+          <t>Do not buy</t>
+        </is>
+      </c>
+      <c r="K13" s="38" t="inlineStr"/>
+      <c r="L13" s="38" t="inlineStr">
+        <is>
+          <t>Rules PDF: 'one but only one module including a microprocessor'; standard-protocol ban</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="95" customHeight="1">
+      <c r="A14" s="38" t="inlineStr">
+        <is>
           <t>EXCLUDE: 915 MHz (US) module variants</t>
         </is>
       </c>
-      <c r="B11" s="38" t="inlineStr">
+      <c r="B14" s="38" t="inlineStr">
         <is>
           <t>902-928 MHz</t>
         </is>
       </c>
-      <c r="C11" s="38" t="inlineStr"/>
-      <c r="D11" s="38" t="inlineStr"/>
-      <c r="E11" s="38" t="inlineStr"/>
-      <c r="F11" s="38" t="inlineStr"/>
-      <c r="G11" s="38" t="inlineStr"/>
-      <c r="H11" s="38" t="inlineStr"/>
-      <c r="I11" s="38" t="inlineStr">
+      <c r="C14" s="38" t="inlineStr"/>
+      <c r="D14" s="38" t="inlineStr"/>
+      <c r="E14" s="38" t="inlineStr"/>
+      <c r="F14" s="38" t="inlineStr"/>
+      <c r="G14" s="38" t="inlineStr"/>
+      <c r="H14" s="38" t="inlineStr"/>
+      <c r="I14" s="38" t="inlineStr">
         <is>
           <t>915-921 MHz is mobile/GSM-R spectrum in Spain (CNAF UN-40), not SRD</t>
         </is>
       </c>
-      <c r="J11" s="38" t="inlineStr">
+      <c r="J14" s="38" t="inlineStr">
         <is>
           <t>Buy 868 variants only</t>
         </is>
       </c>
-      <c r="K11" s="38" t="inlineStr"/>
-      <c r="L11" s="38" t="inlineStr">
+      <c r="K14" s="38" t="inlineStr"/>
+      <c r="L14" s="38" t="inlineStr">
         <is>
           <t>CNAF 2017 (Orden ETU/1033/2017), notas UN - https://www.boe.es/buscar/doc.php?id=BOE-A-2017-12318</t>
         </is>

</xml_diff>